<commit_message>
Aplicar as definições de agosto das lojas Centro e Trancoso
Centro:
- ARIANE e PEDRO deixam de receber comissão
- GENECIR com férias de 01 a 30/08: salário zerado e pendência sobre o
  dia 31/08
- nova aba FOLGUISTAS com as diárias de SERGIO (R$ 150,00) e ANA CELIA
  (R$ 100,00) para o contas a pagar, fora do holerite
- GILSON, UILLIAN e FABIANA marcados como sem comissão

Arraial:
- a comissão da SARA na loja Centro (R$ 2,65) passa a ser somada à folha
  dela, na linha de complemento

Trancoso:
- incentivos confirmados como simples, sem dobrar
- julho havia sido lançado por média; a diferença da comissão dobrada
  será reduzida nas premiações, com observação na linha de prêmio

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_TRANCOSO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_TRANCOSO_pgto_05-09-2026.xlsx
@@ -32,7 +32,7 @@
     <numFmt numFmtId="164" formatCode="R$ #,##0.00;-R$ #,##0.00;&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="19">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -107,12 +107,6 @@
       <name val="Arial"/>
       <color rgb="00008000"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00C00000"/>
-      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -219,7 +213,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -228,7 +222,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -289,28 +283,25 @@
     <xf numFmtId="164" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="14" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="17" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="16" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -677,7 +668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -846,38 +837,30 @@
       <c r="A23" s="4" t="inlineStr"/>
       <c r="B23" s="5" t="inlineStr">
         <is>
+          <t>Os incentivos são simples: entram pelo valor apurado, sem dobrar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Em julho/2026 a comissão foi lançada por média. Com a comissão dobrada a partir de agosto, a empresa vai reduzir nas premiações a diferença.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
           <t>UILLIAN: não recebe comissão sobre vendas (mesmo critério de julho/2026) — a rubrica fica zerada e o apurado dele aparece só na aba BASE.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>PENDÊNCIAS — CONFIRMAR ANTES DE ENVIAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>Horas extras e adicional noturno de agosto (apontamento do ponto).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>Prêmio cota geral e prêmio pré-vencidos, conforme a tabela de metas da loja.</t>
         </is>
       </c>
     </row>
@@ -889,7 +872,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Vales adiantados, convênio e faltas de agosto.</t>
+          <t>Horas extras e adicional noturno de agosto (apontamento do ponto).</t>
         </is>
       </c>
     </row>
@@ -901,7 +884,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Férias, afastamentos e admissões que mudem o salário do mês.</t>
+          <t>Prêmio cota geral e prêmio pré-vencidos, conforme a tabela de metas da loja.</t>
         </is>
       </c>
     </row>
@@ -913,7 +896,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Conferir como as comissões de julho foram efetivamente pagas: a planilha traz o valor simples e o pagamento da loja é em dobro.</t>
+          <t>Vales adiantados, convênio e faltas de agosto.</t>
         </is>
       </c>
     </row>
@@ -925,7 +908,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Confirmar se o dobro vale só para a comissão. Os incentivos estão lançados pelo valor apurado, sem dobrar.</t>
+          <t>Férias, afastamentos e admissões que mudem o salário do mês.</t>
         </is>
       </c>
     </row>
@@ -937,7 +920,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>INIURLE: em julho as horas extras foram lançadas como R$ 442,09, exatamente o mesmo valor do EDEY na loja Arraial — conferir se não houve cópia de célula.</t>
+          <t>Lançar na linha PRÊMIO COTA GERAL o valor já com a redução combinada, para compensar o aumento da comissão dobrada.</t>
         </is>
       </c>
     </row>
@@ -949,37 +932,41 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>INIURLE: em julho as horas extras foram lançadas como R$ 442,09, exatamente o mesmo valor do EDEY na loja Arraial — conferir se não houve cópia de célula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
           <t>UILLIAN também registra vendas no relatório da loja Centro — conferir se alguma comissão deve ser rateada entre as lojas.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO TÉCNICA</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>As células de total e de cálculo são fórmulas. Ao abrir no Excel ou no Google Planilhas elas aparecem calculadas; em visualizadores simples podem aparecer em branco até o arquivo ser aberto.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>ABAS DO ARQUIVO</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -987,7 +974,7 @@
       <c r="A37" s="4" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
+          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -995,7 +982,7 @@
       <c r="A38" s="4" t="inlineStr"/>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
+          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
         </is>
       </c>
     </row>
@@ -1003,7 +990,7 @@
       <c r="A39" s="4" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +998,7 @@
       <c r="A40" s="4" t="inlineStr"/>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>JULHO.26 REVISADO — a folha de julho (TRANCOSO JULHO) reorganizada e conferida.</t>
+          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
         </is>
       </c>
     </row>
@@ -1019,6 +1006,14 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
+          <t>JULHO.26 REVISADO — a folha de julho (TRANCOSO JULHO) reorganizada e conferida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
           <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
         </is>
       </c>
@@ -1026,14 +1021,14 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2016,18 +2011,18 @@
           <t>PRÊMIO COTA GERAL</t>
         </is>
       </c>
-      <c r="B15" s="33" t="n"/>
-      <c r="C15" s="33" t="n"/>
-      <c r="D15" s="33" t="n"/>
-      <c r="E15" s="33" t="n"/>
-      <c r="F15" s="33" t="n"/>
-      <c r="G15" s="20">
+      <c r="B15" s="30" t="n"/>
+      <c r="C15" s="30" t="n"/>
+      <c r="D15" s="30" t="n"/>
+      <c r="E15" s="30" t="n"/>
+      <c r="F15" s="30" t="n"/>
+      <c r="G15" s="31">
         <f>SUM(B15:F15)</f>
         <v/>
       </c>
       <c r="H15" s="32" t="inlineStr">
         <is>
-          <t>PREENCHER conforme a tabela de metas da loja (aba METAS da planilha original).</t>
+          <t>PREENCHER conforme a tabela de metas da loja (aba METAS da planilha original). Lançar já com a redução combinada para compensar o aumento da comissão dobrada.</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2121,7 @@
       </c>
       <c r="H19" s="32" t="inlineStr">
         <is>
-          <t>Incentivo de injetáveis apurado no InovaFarma. NÃO está multiplicado por 2 — confirmar se o dobro vale só para a comissão.</t>
+          <t>Incentivo de injetáveis apurado no InovaFarma. Incentivo é simples: NÃO entra em dobro.</t>
         </is>
       </c>
     </row>
@@ -3400,10 +3395,10 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="26" customHeight="1">
+    <row r="36">
       <c r="A36" s="39" t="inlineStr">
         <is>
-          <t>ATENÇÃO: as comissões desta aba estão pelo valor da planilha (R$ 850,00 do MANOEL, R$ 908,70 do VALDICK etc.), na mesma ordem de grandeza do apurado no sistema. Como o pagamento da loja é o DOBRO da comissão, o líquido revisado acima reproduz a planilha e não o valor efetivamente pago — conferir com a contabilidade como julho foi lançado.</t>
+          <t>OBSERVAÇÃO: em julho/2026 a comissão foi lançada por uma MÉDIA, e não pelo apurado do sistema. A partir de agosto/2026 a loja passa a pagar a comissão em dobro, e a empresa vai reduzir nas premiações a diferença gerada por esse aumento.</t>
         </is>
       </c>
     </row>
@@ -3415,28 +3410,28 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="41" t="inlineStr">
+      <c r="A38" s="39" t="inlineStr">
         <is>
           <t>1. Rubricas separadas em PROVENTOS × DESCONTOS, com subtotais próprios.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="41" t="inlineStr">
+      <c r="A39" s="39" t="inlineStr">
         <is>
           <t>2. Nomes de rubrica padronizados e coluna de observação com a origem de cada valor.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="41" t="inlineStr">
+      <c r="A40" s="39" t="inlineStr">
         <is>
           <t>3. Conferência do DSR: em julho foi usado o fator de agosto (5/26) em vez de 4/27.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="41" t="inlineStr">
+      <c r="A41" s="39" t="inlineStr">
         <is>
           <t>4. Linha de conferência comparando o líquido revisado com o SALDO FINAL da planilha original (tem que fechar em zero).</t>
         </is>
@@ -3535,7 +3530,7 @@
         <f>'HOLERITE AGO.26'!B6</f>
         <v/>
       </c>
-      <c r="E5" s="42" t="n"/>
+      <c r="E5" s="41" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -3557,7 +3552,7 @@
         <f>'HOLERITE AGO.26'!B7</f>
         <v/>
       </c>
-      <c r="E6" s="42" t="n"/>
+      <c r="E6" s="41" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -3579,7 +3574,7 @@
         <f>'HOLERITE AGO.26'!B8</f>
         <v/>
       </c>
-      <c r="E7" s="42" t="n"/>
+      <c r="E7" s="41" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="29" t="inlineStr">
@@ -3601,7 +3596,7 @@
         <f>'HOLERITE AGO.26'!B11</f>
         <v/>
       </c>
-      <c r="E8" s="42" t="n"/>
+      <c r="E8" s="41" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="29" t="inlineStr">
@@ -3623,7 +3618,7 @@
         <f>'HOLERITE AGO.26'!B12</f>
         <v/>
       </c>
-      <c r="E9" s="42" t="n"/>
+      <c r="E9" s="41" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="29" t="inlineStr">
@@ -3645,7 +3640,7 @@
         <f>'HOLERITE AGO.26'!B13</f>
         <v/>
       </c>
-      <c r="E10" s="42" t="n"/>
+      <c r="E10" s="41" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="29" t="inlineStr">
@@ -3667,7 +3662,7 @@
         <f>'HOLERITE AGO.26'!B14</f>
         <v/>
       </c>
-      <c r="E11" s="42" t="n"/>
+      <c r="E11" s="41" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
@@ -3689,7 +3684,7 @@
         <f>'HOLERITE AGO.26'!B15</f>
         <v/>
       </c>
-      <c r="E12" s="42" t="n"/>
+      <c r="E12" s="41" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="29" t="inlineStr">
@@ -3711,7 +3706,7 @@
         <f>'HOLERITE AGO.26'!B16</f>
         <v/>
       </c>
-      <c r="E13" s="42" t="n"/>
+      <c r="E13" s="41" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="29" t="inlineStr">
@@ -3733,7 +3728,7 @@
         <f>'HOLERITE AGO.26'!B17</f>
         <v/>
       </c>
-      <c r="E14" s="42" t="n"/>
+      <c r="E14" s="41" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="29" t="inlineStr">
@@ -3755,7 +3750,7 @@
         <f>'HOLERITE AGO.26'!B18</f>
         <v/>
       </c>
-      <c r="E15" s="42" t="n"/>
+      <c r="E15" s="41" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="29" t="inlineStr">
@@ -3777,7 +3772,7 @@
         <f>'HOLERITE AGO.26'!B19</f>
         <v/>
       </c>
-      <c r="E16" s="42" t="n"/>
+      <c r="E16" s="41" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="29" t="inlineStr">
@@ -3799,7 +3794,7 @@
         <f>'HOLERITE AGO.26'!B20</f>
         <v/>
       </c>
-      <c r="E17" s="42" t="n"/>
+      <c r="E17" s="41" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="29" t="inlineStr">
@@ -3821,25 +3816,25 @@
         <f>'HOLERITE AGO.26'!B21</f>
         <v/>
       </c>
-      <c r="E18" s="42" t="n"/>
+      <c r="E18" s="41" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="43" t="inlineStr">
+      <c r="A19" s="42" t="inlineStr">
         <is>
           <t>UILLIAN</t>
         </is>
       </c>
-      <c r="B19" s="43" t="inlineStr">
+      <c r="B19" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C19" s="43" t="inlineStr">
+      <c r="C19" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D19" s="44">
+      <c r="D19" s="43">
         <f>'HOLERITE AGO.26'!B22</f>
         <v/>
       </c>
@@ -3865,7 +3860,7 @@
         <f>'HOLERITE AGO.26'!B24</f>
         <v/>
       </c>
-      <c r="E20" s="42" t="n"/>
+      <c r="E20" s="41" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="29" t="inlineStr">
@@ -3887,7 +3882,7 @@
         <f>'HOLERITE AGO.26'!B25</f>
         <v/>
       </c>
-      <c r="E21" s="42" t="n"/>
+      <c r="E21" s="41" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
@@ -3909,7 +3904,7 @@
         <f>'HOLERITE AGO.26'!B26</f>
         <v/>
       </c>
-      <c r="E22" s="42" t="n"/>
+      <c r="E22" s="41" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
@@ -3931,7 +3926,7 @@
         <f>'HOLERITE AGO.26'!B27</f>
         <v/>
       </c>
-      <c r="E23" s="42" t="n"/>
+      <c r="E23" s="41" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
@@ -3953,7 +3948,7 @@
         <f>'HOLERITE AGO.26'!B28</f>
         <v/>
       </c>
-      <c r="E24" s="42" t="n"/>
+      <c r="E24" s="41" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
@@ -3975,7 +3970,7 @@
         <f>'HOLERITE AGO.26'!B29</f>
         <v/>
       </c>
-      <c r="E25" s="42" t="n"/>
+      <c r="E25" s="41" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
@@ -3997,51 +3992,51 @@
         <f>'HOLERITE AGO.26'!B30</f>
         <v/>
       </c>
-      <c r="E26" s="42" t="n"/>
+      <c r="E26" s="41" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="43" t="inlineStr">
+      <c r="A27" s="42" t="inlineStr">
         <is>
           <t>UILLIAN</t>
         </is>
       </c>
-      <c r="B27" s="43" t="inlineStr">
+      <c r="B27" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C27" s="43" t="inlineStr">
+      <c r="C27" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D27" s="44">
+      <c r="D27" s="43">
         <f>'HOLERITE AGO.26'!B31</f>
         <v/>
       </c>
       <c r="E27" s="18" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="45" t="inlineStr">
+      <c r="A28" s="44" t="inlineStr">
         <is>
           <t>UILLIAN</t>
         </is>
       </c>
-      <c r="B28" s="46" t="inlineStr">
+      <c r="B28" s="45" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C28" s="46" t="inlineStr">
+      <c r="C28" s="45" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D28" s="47">
+      <c r="D28" s="46">
         <f>'HOLERITE AGO.26'!B33</f>
         <v/>
       </c>
-      <c r="E28" s="48" t="n"/>
+      <c r="E28" s="47" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
@@ -4063,7 +4058,7 @@
         <f>'HOLERITE AGO.26'!C6</f>
         <v/>
       </c>
-      <c r="E30" s="42" t="n"/>
+      <c r="E30" s="41" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="29" t="inlineStr">
@@ -4085,7 +4080,7 @@
         <f>'HOLERITE AGO.26'!C7</f>
         <v/>
       </c>
-      <c r="E31" s="42" t="n"/>
+      <c r="E31" s="41" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
@@ -4107,7 +4102,7 @@
         <f>'HOLERITE AGO.26'!C8</f>
         <v/>
       </c>
-      <c r="E32" s="42" t="n"/>
+      <c r="E32" s="41" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="29" t="inlineStr">
@@ -4129,7 +4124,7 @@
         <f>'HOLERITE AGO.26'!C11</f>
         <v/>
       </c>
-      <c r="E33" s="42" t="n"/>
+      <c r="E33" s="41" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
@@ -4151,7 +4146,7 @@
         <f>'HOLERITE AGO.26'!C12</f>
         <v/>
       </c>
-      <c r="E34" s="42" t="n"/>
+      <c r="E34" s="41" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="29" t="inlineStr">
@@ -4173,7 +4168,7 @@
         <f>'HOLERITE AGO.26'!C13</f>
         <v/>
       </c>
-      <c r="E35" s="42" t="n"/>
+      <c r="E35" s="41" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="29" t="inlineStr">
@@ -4195,7 +4190,7 @@
         <f>'HOLERITE AGO.26'!C14</f>
         <v/>
       </c>
-      <c r="E36" s="42" t="n"/>
+      <c r="E36" s="41" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="29" t="inlineStr">
@@ -4217,7 +4212,7 @@
         <f>'HOLERITE AGO.26'!C15</f>
         <v/>
       </c>
-      <c r="E37" s="42" t="n"/>
+      <c r="E37" s="41" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="29" t="inlineStr">
@@ -4239,7 +4234,7 @@
         <f>'HOLERITE AGO.26'!C16</f>
         <v/>
       </c>
-      <c r="E38" s="42" t="n"/>
+      <c r="E38" s="41" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="29" t="inlineStr">
@@ -4261,7 +4256,7 @@
         <f>'HOLERITE AGO.26'!C17</f>
         <v/>
       </c>
-      <c r="E39" s="42" t="n"/>
+      <c r="E39" s="41" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="29" t="inlineStr">
@@ -4283,7 +4278,7 @@
         <f>'HOLERITE AGO.26'!C18</f>
         <v/>
       </c>
-      <c r="E40" s="42" t="n"/>
+      <c r="E40" s="41" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="29" t="inlineStr">
@@ -4305,7 +4300,7 @@
         <f>'HOLERITE AGO.26'!C19</f>
         <v/>
       </c>
-      <c r="E41" s="42" t="n"/>
+      <c r="E41" s="41" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="29" t="inlineStr">
@@ -4327,7 +4322,7 @@
         <f>'HOLERITE AGO.26'!C20</f>
         <v/>
       </c>
-      <c r="E42" s="42" t="n"/>
+      <c r="E42" s="41" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="29" t="inlineStr">
@@ -4349,25 +4344,25 @@
         <f>'HOLERITE AGO.26'!C21</f>
         <v/>
       </c>
-      <c r="E43" s="42" t="n"/>
+      <c r="E43" s="41" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="43" t="inlineStr">
+      <c r="A44" s="42" t="inlineStr">
         <is>
           <t>MANOEL</t>
         </is>
       </c>
-      <c r="B44" s="43" t="inlineStr">
+      <c r="B44" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C44" s="43" t="inlineStr">
+      <c r="C44" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D44" s="44">
+      <c r="D44" s="43">
         <f>'HOLERITE AGO.26'!C22</f>
         <v/>
       </c>
@@ -4393,7 +4388,7 @@
         <f>'HOLERITE AGO.26'!C24</f>
         <v/>
       </c>
-      <c r="E45" s="42" t="n"/>
+      <c r="E45" s="41" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="29" t="inlineStr">
@@ -4415,7 +4410,7 @@
         <f>'HOLERITE AGO.26'!C25</f>
         <v/>
       </c>
-      <c r="E46" s="42" t="n"/>
+      <c r="E46" s="41" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="29" t="inlineStr">
@@ -4437,7 +4432,7 @@
         <f>'HOLERITE AGO.26'!C26</f>
         <v/>
       </c>
-      <c r="E47" s="42" t="n"/>
+      <c r="E47" s="41" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="29" t="inlineStr">
@@ -4459,7 +4454,7 @@
         <f>'HOLERITE AGO.26'!C27</f>
         <v/>
       </c>
-      <c r="E48" s="42" t="n"/>
+      <c r="E48" s="41" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="29" t="inlineStr">
@@ -4481,7 +4476,7 @@
         <f>'HOLERITE AGO.26'!C28</f>
         <v/>
       </c>
-      <c r="E49" s="42" t="n"/>
+      <c r="E49" s="41" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="29" t="inlineStr">
@@ -4503,7 +4498,7 @@
         <f>'HOLERITE AGO.26'!C29</f>
         <v/>
       </c>
-      <c r="E50" s="42" t="n"/>
+      <c r="E50" s="41" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="29" t="inlineStr">
@@ -4525,51 +4520,51 @@
         <f>'HOLERITE AGO.26'!C30</f>
         <v/>
       </c>
-      <c r="E51" s="42" t="n"/>
+      <c r="E51" s="41" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="43" t="inlineStr">
+      <c r="A52" s="42" t="inlineStr">
         <is>
           <t>MANOEL</t>
         </is>
       </c>
-      <c r="B52" s="43" t="inlineStr">
+      <c r="B52" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C52" s="43" t="inlineStr">
+      <c r="C52" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D52" s="44">
+      <c r="D52" s="43">
         <f>'HOLERITE AGO.26'!C31</f>
         <v/>
       </c>
       <c r="E52" s="18" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="45" t="inlineStr">
+      <c r="A53" s="44" t="inlineStr">
         <is>
           <t>MANOEL</t>
         </is>
       </c>
-      <c r="B53" s="46" t="inlineStr">
+      <c r="B53" s="45" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C53" s="46" t="inlineStr">
+      <c r="C53" s="45" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D53" s="47">
+      <c r="D53" s="46">
         <f>'HOLERITE AGO.26'!C33</f>
         <v/>
       </c>
-      <c r="E53" s="48" t="n"/>
+      <c r="E53" s="47" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="29" t="inlineStr">
@@ -4591,7 +4586,7 @@
         <f>'HOLERITE AGO.26'!D6</f>
         <v/>
       </c>
-      <c r="E55" s="42" t="n"/>
+      <c r="E55" s="41" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="29" t="inlineStr">
@@ -4613,7 +4608,7 @@
         <f>'HOLERITE AGO.26'!D7</f>
         <v/>
       </c>
-      <c r="E56" s="42" t="n"/>
+      <c r="E56" s="41" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="29" t="inlineStr">
@@ -4635,7 +4630,7 @@
         <f>'HOLERITE AGO.26'!D8</f>
         <v/>
       </c>
-      <c r="E57" s="42" t="n"/>
+      <c r="E57" s="41" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="29" t="inlineStr">
@@ -4657,7 +4652,7 @@
         <f>'HOLERITE AGO.26'!D11</f>
         <v/>
       </c>
-      <c r="E58" s="42" t="n"/>
+      <c r="E58" s="41" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="29" t="inlineStr">
@@ -4679,7 +4674,7 @@
         <f>'HOLERITE AGO.26'!D12</f>
         <v/>
       </c>
-      <c r="E59" s="42" t="n"/>
+      <c r="E59" s="41" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="29" t="inlineStr">
@@ -4701,7 +4696,7 @@
         <f>'HOLERITE AGO.26'!D13</f>
         <v/>
       </c>
-      <c r="E60" s="42" t="n"/>
+      <c r="E60" s="41" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="29" t="inlineStr">
@@ -4723,7 +4718,7 @@
         <f>'HOLERITE AGO.26'!D14</f>
         <v/>
       </c>
-      <c r="E61" s="42" t="n"/>
+      <c r="E61" s="41" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="29" t="inlineStr">
@@ -4745,7 +4740,7 @@
         <f>'HOLERITE AGO.26'!D15</f>
         <v/>
       </c>
-      <c r="E62" s="42" t="n"/>
+      <c r="E62" s="41" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="29" t="inlineStr">
@@ -4767,7 +4762,7 @@
         <f>'HOLERITE AGO.26'!D16</f>
         <v/>
       </c>
-      <c r="E63" s="42" t="n"/>
+      <c r="E63" s="41" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="29" t="inlineStr">
@@ -4789,7 +4784,7 @@
         <f>'HOLERITE AGO.26'!D17</f>
         <v/>
       </c>
-      <c r="E64" s="42" t="n"/>
+      <c r="E64" s="41" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="29" t="inlineStr">
@@ -4811,7 +4806,7 @@
         <f>'HOLERITE AGO.26'!D18</f>
         <v/>
       </c>
-      <c r="E65" s="42" t="n"/>
+      <c r="E65" s="41" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="29" t="inlineStr">
@@ -4833,7 +4828,7 @@
         <f>'HOLERITE AGO.26'!D19</f>
         <v/>
       </c>
-      <c r="E66" s="42" t="n"/>
+      <c r="E66" s="41" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="29" t="inlineStr">
@@ -4855,7 +4850,7 @@
         <f>'HOLERITE AGO.26'!D20</f>
         <v/>
       </c>
-      <c r="E67" s="42" t="n"/>
+      <c r="E67" s="41" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="29" t="inlineStr">
@@ -4877,25 +4872,25 @@
         <f>'HOLERITE AGO.26'!D21</f>
         <v/>
       </c>
-      <c r="E68" s="42" t="n"/>
+      <c r="E68" s="41" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="43" t="inlineStr">
+      <c r="A69" s="42" t="inlineStr">
         <is>
           <t>VALDICK</t>
         </is>
       </c>
-      <c r="B69" s="43" t="inlineStr">
+      <c r="B69" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C69" s="43" t="inlineStr">
+      <c r="C69" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D69" s="44">
+      <c r="D69" s="43">
         <f>'HOLERITE AGO.26'!D22</f>
         <v/>
       </c>
@@ -4921,7 +4916,7 @@
         <f>'HOLERITE AGO.26'!D24</f>
         <v/>
       </c>
-      <c r="E70" s="42" t="n"/>
+      <c r="E70" s="41" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="29" t="inlineStr">
@@ -4943,7 +4938,7 @@
         <f>'HOLERITE AGO.26'!D25</f>
         <v/>
       </c>
-      <c r="E71" s="42" t="n"/>
+      <c r="E71" s="41" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="29" t="inlineStr">
@@ -4965,7 +4960,7 @@
         <f>'HOLERITE AGO.26'!D26</f>
         <v/>
       </c>
-      <c r="E72" s="42" t="n"/>
+      <c r="E72" s="41" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="29" t="inlineStr">
@@ -4987,7 +4982,7 @@
         <f>'HOLERITE AGO.26'!D27</f>
         <v/>
       </c>
-      <c r="E73" s="42" t="n"/>
+      <c r="E73" s="41" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="29" t="inlineStr">
@@ -5009,7 +5004,7 @@
         <f>'HOLERITE AGO.26'!D28</f>
         <v/>
       </c>
-      <c r="E74" s="42" t="n"/>
+      <c r="E74" s="41" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="29" t="inlineStr">
@@ -5031,7 +5026,7 @@
         <f>'HOLERITE AGO.26'!D29</f>
         <v/>
       </c>
-      <c r="E75" s="42" t="n"/>
+      <c r="E75" s="41" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="29" t="inlineStr">
@@ -5053,51 +5048,51 @@
         <f>'HOLERITE AGO.26'!D30</f>
         <v/>
       </c>
-      <c r="E76" s="42" t="n"/>
+      <c r="E76" s="41" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="43" t="inlineStr">
+      <c r="A77" s="42" t="inlineStr">
         <is>
           <t>VALDICK</t>
         </is>
       </c>
-      <c r="B77" s="43" t="inlineStr">
+      <c r="B77" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C77" s="43" t="inlineStr">
+      <c r="C77" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D77" s="44">
+      <c r="D77" s="43">
         <f>'HOLERITE AGO.26'!D31</f>
         <v/>
       </c>
       <c r="E77" s="18" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="45" t="inlineStr">
+      <c r="A78" s="44" t="inlineStr">
         <is>
           <t>VALDICK</t>
         </is>
       </c>
-      <c r="B78" s="46" t="inlineStr">
+      <c r="B78" s="45" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C78" s="46" t="inlineStr">
+      <c r="C78" s="45" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D78" s="47">
+      <c r="D78" s="46">
         <f>'HOLERITE AGO.26'!D33</f>
         <v/>
       </c>
-      <c r="E78" s="48" t="n"/>
+      <c r="E78" s="47" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="29" t="inlineStr">
@@ -5119,7 +5114,7 @@
         <f>'HOLERITE AGO.26'!E6</f>
         <v/>
       </c>
-      <c r="E80" s="42" t="n"/>
+      <c r="E80" s="41" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="29" t="inlineStr">
@@ -5141,7 +5136,7 @@
         <f>'HOLERITE AGO.26'!E7</f>
         <v/>
       </c>
-      <c r="E81" s="42" t="n"/>
+      <c r="E81" s="41" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="29" t="inlineStr">
@@ -5163,7 +5158,7 @@
         <f>'HOLERITE AGO.26'!E8</f>
         <v/>
       </c>
-      <c r="E82" s="42" t="n"/>
+      <c r="E82" s="41" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="29" t="inlineStr">
@@ -5185,7 +5180,7 @@
         <f>'HOLERITE AGO.26'!E11</f>
         <v/>
       </c>
-      <c r="E83" s="42" t="n"/>
+      <c r="E83" s="41" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="29" t="inlineStr">
@@ -5207,7 +5202,7 @@
         <f>'HOLERITE AGO.26'!E12</f>
         <v/>
       </c>
-      <c r="E84" s="42" t="n"/>
+      <c r="E84" s="41" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="29" t="inlineStr">
@@ -5229,7 +5224,7 @@
         <f>'HOLERITE AGO.26'!E13</f>
         <v/>
       </c>
-      <c r="E85" s="42" t="n"/>
+      <c r="E85" s="41" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="29" t="inlineStr">
@@ -5251,7 +5246,7 @@
         <f>'HOLERITE AGO.26'!E14</f>
         <v/>
       </c>
-      <c r="E86" s="42" t="n"/>
+      <c r="E86" s="41" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="29" t="inlineStr">
@@ -5273,7 +5268,7 @@
         <f>'HOLERITE AGO.26'!E15</f>
         <v/>
       </c>
-      <c r="E87" s="42" t="n"/>
+      <c r="E87" s="41" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="29" t="inlineStr">
@@ -5295,7 +5290,7 @@
         <f>'HOLERITE AGO.26'!E16</f>
         <v/>
       </c>
-      <c r="E88" s="42" t="n"/>
+      <c r="E88" s="41" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="29" t="inlineStr">
@@ -5317,7 +5312,7 @@
         <f>'HOLERITE AGO.26'!E17</f>
         <v/>
       </c>
-      <c r="E89" s="42" t="n"/>
+      <c r="E89" s="41" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="29" t="inlineStr">
@@ -5339,7 +5334,7 @@
         <f>'HOLERITE AGO.26'!E18</f>
         <v/>
       </c>
-      <c r="E90" s="42" t="n"/>
+      <c r="E90" s="41" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="29" t="inlineStr">
@@ -5361,7 +5356,7 @@
         <f>'HOLERITE AGO.26'!E19</f>
         <v/>
       </c>
-      <c r="E91" s="42" t="n"/>
+      <c r="E91" s="41" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="29" t="inlineStr">
@@ -5383,7 +5378,7 @@
         <f>'HOLERITE AGO.26'!E20</f>
         <v/>
       </c>
-      <c r="E92" s="42" t="n"/>
+      <c r="E92" s="41" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="29" t="inlineStr">
@@ -5405,25 +5400,25 @@
         <f>'HOLERITE AGO.26'!E21</f>
         <v/>
       </c>
-      <c r="E93" s="42" t="n"/>
+      <c r="E93" s="41" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="43" t="inlineStr">
+      <c r="A94" s="42" t="inlineStr">
         <is>
           <t>INIURLE</t>
         </is>
       </c>
-      <c r="B94" s="43" t="inlineStr">
+      <c r="B94" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C94" s="43" t="inlineStr">
+      <c r="C94" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D94" s="44">
+      <c r="D94" s="43">
         <f>'HOLERITE AGO.26'!E22</f>
         <v/>
       </c>
@@ -5449,7 +5444,7 @@
         <f>'HOLERITE AGO.26'!E24</f>
         <v/>
       </c>
-      <c r="E95" s="42" t="n"/>
+      <c r="E95" s="41" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="29" t="inlineStr">
@@ -5471,7 +5466,7 @@
         <f>'HOLERITE AGO.26'!E25</f>
         <v/>
       </c>
-      <c r="E96" s="42" t="n"/>
+      <c r="E96" s="41" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="29" t="inlineStr">
@@ -5493,7 +5488,7 @@
         <f>'HOLERITE AGO.26'!E26</f>
         <v/>
       </c>
-      <c r="E97" s="42" t="n"/>
+      <c r="E97" s="41" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="29" t="inlineStr">
@@ -5515,7 +5510,7 @@
         <f>'HOLERITE AGO.26'!E27</f>
         <v/>
       </c>
-      <c r="E98" s="42" t="n"/>
+      <c r="E98" s="41" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="29" t="inlineStr">
@@ -5537,7 +5532,7 @@
         <f>'HOLERITE AGO.26'!E28</f>
         <v/>
       </c>
-      <c r="E99" s="42" t="n"/>
+      <c r="E99" s="41" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="29" t="inlineStr">
@@ -5559,7 +5554,7 @@
         <f>'HOLERITE AGO.26'!E29</f>
         <v/>
       </c>
-      <c r="E100" s="42" t="n"/>
+      <c r="E100" s="41" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="29" t="inlineStr">
@@ -5581,51 +5576,51 @@
         <f>'HOLERITE AGO.26'!E30</f>
         <v/>
       </c>
-      <c r="E101" s="42" t="n"/>
+      <c r="E101" s="41" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="43" t="inlineStr">
+      <c r="A102" s="42" t="inlineStr">
         <is>
           <t>INIURLE</t>
         </is>
       </c>
-      <c r="B102" s="43" t="inlineStr">
+      <c r="B102" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C102" s="43" t="inlineStr">
+      <c r="C102" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D102" s="44">
+      <c r="D102" s="43">
         <f>'HOLERITE AGO.26'!E31</f>
         <v/>
       </c>
       <c r="E102" s="18" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="45" t="inlineStr">
+      <c r="A103" s="44" t="inlineStr">
         <is>
           <t>INIURLE</t>
         </is>
       </c>
-      <c r="B103" s="46" t="inlineStr">
+      <c r="B103" s="45" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C103" s="46" t="inlineStr">
+      <c r="C103" s="45" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D103" s="47">
+      <c r="D103" s="46">
         <f>'HOLERITE AGO.26'!E33</f>
         <v/>
       </c>
-      <c r="E103" s="48" t="n"/>
+      <c r="E103" s="47" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="29" t="inlineStr">
@@ -5647,7 +5642,7 @@
         <f>'HOLERITE AGO.26'!F6</f>
         <v/>
       </c>
-      <c r="E105" s="42" t="n"/>
+      <c r="E105" s="41" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="29" t="inlineStr">
@@ -5669,7 +5664,7 @@
         <f>'HOLERITE AGO.26'!F7</f>
         <v/>
       </c>
-      <c r="E106" s="42" t="n"/>
+      <c r="E106" s="41" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="29" t="inlineStr">
@@ -5691,7 +5686,7 @@
         <f>'HOLERITE AGO.26'!F8</f>
         <v/>
       </c>
-      <c r="E107" s="42" t="n"/>
+      <c r="E107" s="41" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="29" t="inlineStr">
@@ -5713,7 +5708,7 @@
         <f>'HOLERITE AGO.26'!F11</f>
         <v/>
       </c>
-      <c r="E108" s="42" t="n"/>
+      <c r="E108" s="41" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="29" t="inlineStr">
@@ -5735,7 +5730,7 @@
         <f>'HOLERITE AGO.26'!F12</f>
         <v/>
       </c>
-      <c r="E109" s="42" t="n"/>
+      <c r="E109" s="41" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="29" t="inlineStr">
@@ -5757,7 +5752,7 @@
         <f>'HOLERITE AGO.26'!F13</f>
         <v/>
       </c>
-      <c r="E110" s="42" t="n"/>
+      <c r="E110" s="41" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="29" t="inlineStr">
@@ -5779,7 +5774,7 @@
         <f>'HOLERITE AGO.26'!F14</f>
         <v/>
       </c>
-      <c r="E111" s="42" t="n"/>
+      <c r="E111" s="41" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="29" t="inlineStr">
@@ -5801,7 +5796,7 @@
         <f>'HOLERITE AGO.26'!F15</f>
         <v/>
       </c>
-      <c r="E112" s="42" t="n"/>
+      <c r="E112" s="41" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="29" t="inlineStr">
@@ -5823,7 +5818,7 @@
         <f>'HOLERITE AGO.26'!F16</f>
         <v/>
       </c>
-      <c r="E113" s="42" t="n"/>
+      <c r="E113" s="41" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="29" t="inlineStr">
@@ -5845,7 +5840,7 @@
         <f>'HOLERITE AGO.26'!F17</f>
         <v/>
       </c>
-      <c r="E114" s="42" t="n"/>
+      <c r="E114" s="41" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="29" t="inlineStr">
@@ -5867,7 +5862,7 @@
         <f>'HOLERITE AGO.26'!F18</f>
         <v/>
       </c>
-      <c r="E115" s="42" t="n"/>
+      <c r="E115" s="41" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="29" t="inlineStr">
@@ -5889,7 +5884,7 @@
         <f>'HOLERITE AGO.26'!F19</f>
         <v/>
       </c>
-      <c r="E116" s="42" t="n"/>
+      <c r="E116" s="41" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="29" t="inlineStr">
@@ -5911,7 +5906,7 @@
         <f>'HOLERITE AGO.26'!F20</f>
         <v/>
       </c>
-      <c r="E117" s="42" t="n"/>
+      <c r="E117" s="41" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="29" t="inlineStr">
@@ -5933,25 +5928,25 @@
         <f>'HOLERITE AGO.26'!F21</f>
         <v/>
       </c>
-      <c r="E118" s="42" t="n"/>
+      <c r="E118" s="41" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="43" t="inlineStr">
+      <c r="A119" s="42" t="inlineStr">
         <is>
           <t>TAMILES</t>
         </is>
       </c>
-      <c r="B119" s="43" t="inlineStr">
+      <c r="B119" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C119" s="43" t="inlineStr">
+      <c r="C119" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D119" s="44">
+      <c r="D119" s="43">
         <f>'HOLERITE AGO.26'!F22</f>
         <v/>
       </c>
@@ -5977,7 +5972,7 @@
         <f>'HOLERITE AGO.26'!F24</f>
         <v/>
       </c>
-      <c r="E120" s="42" t="n"/>
+      <c r="E120" s="41" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="29" t="inlineStr">
@@ -5999,7 +5994,7 @@
         <f>'HOLERITE AGO.26'!F25</f>
         <v/>
       </c>
-      <c r="E121" s="42" t="n"/>
+      <c r="E121" s="41" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="29" t="inlineStr">
@@ -6021,7 +6016,7 @@
         <f>'HOLERITE AGO.26'!F26</f>
         <v/>
       </c>
-      <c r="E122" s="42" t="n"/>
+      <c r="E122" s="41" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="29" t="inlineStr">
@@ -6043,7 +6038,7 @@
         <f>'HOLERITE AGO.26'!F27</f>
         <v/>
       </c>
-      <c r="E123" s="42" t="n"/>
+      <c r="E123" s="41" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="29" t="inlineStr">
@@ -6065,7 +6060,7 @@
         <f>'HOLERITE AGO.26'!F28</f>
         <v/>
       </c>
-      <c r="E124" s="42" t="n"/>
+      <c r="E124" s="41" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="29" t="inlineStr">
@@ -6087,7 +6082,7 @@
         <f>'HOLERITE AGO.26'!F29</f>
         <v/>
       </c>
-      <c r="E125" s="42" t="n"/>
+      <c r="E125" s="41" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="29" t="inlineStr">
@@ -6109,51 +6104,51 @@
         <f>'HOLERITE AGO.26'!F30</f>
         <v/>
       </c>
-      <c r="E126" s="42" t="n"/>
+      <c r="E126" s="41" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="43" t="inlineStr">
+      <c r="A127" s="42" t="inlineStr">
         <is>
           <t>TAMILES</t>
         </is>
       </c>
-      <c r="B127" s="43" t="inlineStr">
+      <c r="B127" s="42" t="inlineStr">
         <is>
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C127" s="43" t="inlineStr">
+      <c r="C127" s="42" t="inlineStr">
         <is>
           <t>Subtotal</t>
         </is>
       </c>
-      <c r="D127" s="44">
+      <c r="D127" s="43">
         <f>'HOLERITE AGO.26'!F31</f>
         <v/>
       </c>
       <c r="E127" s="18" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="45" t="inlineStr">
+      <c r="A128" s="44" t="inlineStr">
         <is>
           <t>TAMILES</t>
         </is>
       </c>
-      <c r="B128" s="46" t="inlineStr">
+      <c r="B128" s="45" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER</t>
         </is>
       </c>
-      <c r="C128" s="46" t="inlineStr">
+      <c r="C128" s="45" t="inlineStr">
         <is>
           <t>Líquido</t>
         </is>
       </c>
-      <c r="D128" s="47">
+      <c r="D128" s="46">
         <f>'HOLERITE AGO.26'!F33</f>
         <v/>
       </c>
-      <c r="E128" s="48" t="n"/>
+      <c r="E128" s="47" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:E128"/>
@@ -6195,12 +6190,12 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="49" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>Escolha o colaborador:</t>
         </is>
       </c>
-      <c r="C4" s="50" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>UILLIAN</t>
         </is>
@@ -6380,7 +6375,7 @@
           <t>TOTAL DE PROVENTOS</t>
         </is>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="43">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$22:$F$22,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$F$4,0)),0)</f>
         <v/>
       </c>
@@ -6477,7 +6472,7 @@
           <t>TOTAL DE DESCONTOS</t>
         </is>
       </c>
-      <c r="C30" s="44">
+      <c r="C30" s="43">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$31:$F$31,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$F$4,0)),0)</f>
         <v/>
       </c>
@@ -6492,18 +6487,18 @@
       <c r="D31" s="28" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="51" t="inlineStr">
+      <c r="B32" s="50" t="inlineStr">
         <is>
           <t>LÍQUIDO A RECEBER EM 05/09/2026</t>
         </is>
       </c>
-      <c r="C32" s="52">
+      <c r="C32" s="51">
         <f>IFERROR(INDEX('HOLERITE AGO.26'!$B$33:$F$33,1,MATCH($C$4,'HOLERITE AGO.26'!$B$4:$F$4,0)),0)</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="53" t="inlineStr">
+      <c r="B34" s="52" t="inlineStr">
         <is>
           <t>Vendas do colaborador no mês (InovaFarma):</t>
         </is>

</xml_diff>

<commit_message>
Registrar o atestado da TAMILES para a competência de setembro
Atestado de 7 dias entregue em 02/09/2026 (02/09 a 08/09). Como é
setembro, não afeta a folha de agosto: fica registrado num bloco de
ocorrências da próxima competência na aba PONTO AGO.26 do Trancoso e na
lista de pendências da capa.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N2n4hj3F39Ez9XRrPSJYG5
</commit_message>
<xml_diff>
--- a/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_TRANCOSO_pgto_05-09-2026.xlsx
+++ b/relatorios/contabilidade/RELATORIO_HOLERITE_AGOSTO_2026_TRANCOSO_pgto_05-09-2026.xlsx
@@ -215,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -307,6 +307,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -672,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -924,7 +927,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Lançar na linha PRÊMIO COTA GERAL o valor já com a redução combinada, para compensar o aumento da comissão dobrada.</t>
+          <t>TAMILES: atestado de 02/09 a 08/09/2026 — lançar na folha de SETEMBRO como falta justificada (abonada), sem desconto. Não entra nesta folha de agosto.</t>
         </is>
       </c>
     </row>
@@ -936,37 +939,41 @@
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
+          <t>Lançar na linha PRÊMIO COTA GERAL o valor já com a redução combinada, para compensar o aumento da comissão dobrada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="17" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
           <t>UILLIAN também registra vendas no relatório da loja Centro — conferir se alguma comissão deve ser rateada entre as lojas.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>OBSERVAÇÃO TÉCNICA</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="17" customHeight="1">
-      <c r="A34" s="4" t="inlineStr"/>
-      <c r="B34" s="5" t="inlineStr">
+    <row r="35" ht="17" customHeight="1">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>As células de total e de cálculo são fórmulas. Ao abrir no Excel ou no Google Planilhas elas aparecem calculadas; em visualizadores simples podem aparecer em branco até o arquivo ser aberto.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="20" customHeight="1">
-      <c r="A35" s="3" t="inlineStr">
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>ABAS DO ARQUIVO</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="17" customHeight="1">
-      <c r="A36" s="4" t="inlineStr"/>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -974,7 +981,7 @@
       <c r="A37" s="4" t="inlineStr"/>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
+          <t>HOLERITE AGO.26 — relatório principal da competência agosto/2026.</t>
         </is>
       </c>
     </row>
@@ -982,7 +989,7 @@
       <c r="A38" s="4" t="inlineStr"/>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
+          <t>GANHOS DO COLABORADOR — demonstrativo individual, pronto para imprimir/mandar.</t>
         </is>
       </c>
     </row>
@@ -990,7 +997,7 @@
       <c r="A39" s="4" t="inlineStr"/>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
+          <t>LISTA CONTABILIDADE — os mesmos lançamentos em formato de lista.</t>
         </is>
       </c>
     </row>
@@ -998,7 +1005,7 @@
       <c r="A40" s="4" t="inlineStr"/>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>JULHO.26 REVISADO — a folha de julho (TRANCOSO JULHO) reorganizada e conferida.</t>
+          <t>BASE INOVAFARMA AGO.26 — apuração de comissões e incentivos por vendedor.</t>
         </is>
       </c>
     </row>
@@ -1006,13 +1013,21 @@
       <c r="A41" s="4" t="inlineStr"/>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
+          <t>JULHO.26 REVISADO — a folha de julho (TRANCOSO JULHO) reorganizada e conferida.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="17" customHeight="1">
       <c r="A42" s="4" t="inlineStr"/>
       <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>PARÂMETROS — calendário do mês, fator do DSR e valores fixos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="17" customHeight="1">
+      <c r="A43" s="4" t="inlineStr"/>
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>PONTO AGO.26 — horas extras, adicional noturno e feriado trabalhado; alimenta o holerite.</t>
         </is>
@@ -1024,11 +1039,11 @@
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A21:B21"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A36:B36"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6698,7 +6713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6997,14 +7012,50 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="19" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>OCORRÊNCIAS PARA A PRÓXIMA COMPETÊNCIA (SETEMBRO/2026) — NÃO ENTRAM NESTA FOLHA</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="n"/>
+      <c r="C21" s="28" t="n"/>
+      <c r="D21" s="28" t="n"/>
+      <c r="E21" s="28" t="n"/>
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="n"/>
+      <c r="H21" s="28" t="n"/>
+      <c r="I21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>TAMILES</t>
+        </is>
+      </c>
+      <c r="B22" s="55" t="inlineStr">
+        <is>
+          <t>Atestado médico de 7 dias, entregue em 02/09/2026 — cobre de 02/09 a 08/09/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Cai na competência SETEMBRO/2026 (holerite pago em 05/10/2026), não nesta folha de agosto. Atestado de até 15 dias é abonado pela empresa: falta justificada, sem desconto de salário nem de DSR. A partir do 16º dia seria auxílio-doença pelo INSS. Anexar o atestado à pasta da funcionária.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:I13"/>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A19:I19"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A17:I17"/>
     <mergeCell ref="A18:I18"/>
+    <mergeCell ref="B22:I22"/>
+    <mergeCell ref="B23:I23"/>
     <mergeCell ref="A16:I16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>